<commit_message>
Update all Quizizz spreadsheets with dynamic question types (Multiple, Multiple Choice, Boolean) per docx content
</commit_message>
<xml_diff>
--- a/Paket_10_Bahasa_Indonesia_TKA_SD.xlsx
+++ b/Paket_10_Bahasa_Indonesia_TKA_SD.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Paket 10 Bahasa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,27 +471,27 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 1: contoh soal pemahaman teks.</t>
+          <t>Bacalah teks berikut! 'Kebun Raya Bogor didirikan pada tahun 1817 atas gagasan Prof. C.G.C. Reinwardt. Di dalam kebun botani seluas puluhan hektare ini terdapat ribuan koleksi jenis pohon dan tanaman langka dari berbagai belahan dunia.' Pernyataan manakah yang sesuai dengan teks tersebut?</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Kebun Raya Bogor didirikan di pulau Bali pada tahun 1900</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. Prof. C.G.C. Reinwardt adalah tokoh pencetus gagasan pendirian Kebun Raya Bogor</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Di dalam Kebun Raya Bogor hanya terdapat tanaman kelapa sawit</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Kebun Raya Bogor dikelola langsung oleh pemerintah luar negeri</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -502,7 +502,11 @@
       <c r="H2" t="n">
         <v>60</v>
       </c>
-      <c r="I2" t="inlineStr"/>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -512,27 +516,27 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 2: contoh soal pemahaman teks.</t>
+          <t>Bacalah paragraf berikut! 'Pendidikan karakter sangat penting ditanamkan kepada anak-anak sejak usia dini. Melalui pendidikan karakter, anak-anak tidak hanya menjadi cerdas secara intelektual, tetapi juga memiliki integritas, kejujuran, serta kepedulian sosial yang tinggi terhadap sesama warga masyarakat.' Ide pokok paragraf tersebut adalah...</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Kecerdasan intelektual anak sekolah di kota besar</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. Pentingnya penanaman pendidikan karakter sejak usia dini</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Cara mendirikan sekolah unggulan berbasis karakter bangsa</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Kegiatan sosial masyarakat di lingkungan tempat tinggal</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -543,7 +547,11 @@
       <c r="H3" t="n">
         <v>60</v>
       </c>
-      <c r="I3" t="inlineStr"/>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -553,27 +561,27 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 3: contoh soal pemahaman teks.</t>
+          <t>Bacalah kalimat berikut! 'Para transmigran asal Jawa Tengah itu mendapat alokasi lahan pertanian subur di wilayah Sulawesi.' Apakah makna kata 'alokasi' dalam kalimat tersebut?</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Peninjauan atau pengawasan berkala</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. Penjatahan atau penyediaan sesuatu untuk tujuan tertentu</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Pemindahan penduduk antarpulau</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Penggusuran lahan pemukiman warga</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -584,7 +592,11 @@
       <c r="H4" t="n">
         <v>60</v>
       </c>
-      <c r="I4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -594,27 +606,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 4: contoh soal pemahaman teks.</t>
+          <t>Bacalah pantun berikut! Bunga melati harum warnanya, Tumbuh subur di taman kota. Bekerja keraslah dengan rencana, Agar tercapai cita-cita. Pesan yang terkandung dalam pantun tersebut adalah...</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Kita harus merawat bunga melati di taman</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. Menanam bunga membuat taman menjadi harum</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Kita harus bekerja keras dengan terencana demi meraih cita-cita</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Cita-cita tinggi hanya dicapai oleh orang pemalas</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -625,17 +637,21 @@
       <c r="H5" t="n">
         <v>60</v>
       </c>
-      <c r="I5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 5: contoh soal pemahaman teks.</t>
+          <t>Bacalah kutipan cerita berikut! 'Meskipun lelah setelah bekerja seharian di ladang, Ibu selalu menyempatkan diri mendengarkan keluh kesah Rani sambil membelai rambutnya dengan penuh kelembutan.' Manakah pernyataan yang BENAR? (Jawaban benar lebih dari satu) ☐ A. Tokoh Ibu memiliki sifat yang penyayang dan penuh perhatian ☐ B. Tokoh Rani digambarkan sebagai anak yang tidak peduli kepada orang tua ☐ C. Latar suasana dalam kutipan cerita tersebut penuh kehangatan keluarga ☐ D. Amanat cerita adalah kita harus menyayangi orang tua yang bekerja keras [Pilihan Ganda Kompleks: Jawaban benar lebih dari satu]</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -666,7 +682,11 @@
       <c r="H6" t="n">
         <v>60</v>
       </c>
-      <c r="I6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -676,27 +696,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 6: contoh soal pemahaman teks.</t>
+          <t>Kalimat berikut yang menggunakan ejaan dan kata baku yang tepat adalah...</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Apotik di ujung jalan itu menjual obat generik berkwalitas</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. Apotek di ujung jalan itu menjual obat generik berkualitas</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Apotik di ujung jalan itu menjual obat generik berkualitas</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Apotek di ujung jalan itu menjual obat generik berkwalitas</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -707,17 +727,21 @@
       <c r="H7" t="n">
         <v>60</v>
       </c>
-      <c r="I7" t="inlineStr"/>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 7: contoh soal pemahaman teks.</t>
+          <t>Bacalah teks informasi berikut! 'Harimau sumatera (Panthera tigris sumatrae) merupakan salah satu subspesies harimau langka yang kini hanya dapat ditemukan di pulau Sumatra. Habitat aslinya di hutan tropis terancam oleh perburuan liar dan pembukaan lahan.' Tentukan kebenaran pernyataan berikut! [Pilihan Ganda Kompleks: Kategori Benar / Salah]</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -748,7 +772,11 @@
       <c r="H8" t="n">
         <v>60</v>
       </c>
-      <c r="I8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -758,27 +786,27 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 8: contoh soal pemahaman teks.</t>
+          <t>Sinonim dari kata 'inovasi' dalam kalimat pengembangan iptek adalah...</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. pembaharuan</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. peniruan</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. kerusakan</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. penundaan</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -789,7 +817,11 @@
       <c r="H9" t="n">
         <v>60</v>
       </c>
-      <c r="I9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -799,27 +831,27 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 9: contoh soal pemahaman teks.</t>
+          <t>Susunan kalimat petunjuk mencuci tangan yang benar: (1) Basahi tangan dengan air bersih mengalir. (2) Gosok telapak tangan, punggung tangan, dan sela-sela jari. (3) Tuangkan sabun cair secukupnya pada telapak tangan. (4) Bilas dengan air bersih lalu keringkan dengan handuk. Urutan yang padu adalah...</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. (1) - (3) - (2) - (4)</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. (3) - (1) - (2) - (4)</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. (1) - (2) - (3) - (4)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. (3) - (2) - (1) - (4)</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -830,7 +862,11 @@
       <c r="H10" t="n">
         <v>60</v>
       </c>
-      <c r="I10" t="inlineStr"/>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -840,27 +876,27 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 10: contoh soal pemahaman teks.</t>
+          <t>Penulisan nama dan gelar yang benar adalah...</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Dr. H. Moh. Hatta, M.Pd.</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. dr. h. moh. hatta, m.pd</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Dokter H. Moh. Hatta</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Dr h Moh Hatta Mpd</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -871,7 +907,11 @@
       <c r="H11" t="n">
         <v>60</v>
       </c>
-      <c r="I11" t="inlineStr"/>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -881,27 +921,27 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 11: contoh soal pemahaman teks.</t>
+          <t>Teks nonfiksi tentang manfaat lidah buaya menyebutkan bahwa gel daun lidah buaya berkhasiat menyembuhkan luka bakar ringan dan melembabkan kulit. Informasi tersebut adalah...</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. Manfaat lidah buaya untuk bidang otomotif</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. Khasiat lidah buaya untuk kesehatan dan kecantikan kulit</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. Cara menanam lidah buaya di pot gantung</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. Bahaya getah lidah buaya bagi kesehatan</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -912,17 +952,21 @@
       <c r="H12" t="n">
         <v>60</v>
       </c>
-      <c r="I12" t="inlineStr"/>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 12: contoh soal pemahaman teks.</t>
+          <t>Ilustrasi: 'Rian selalu menjadi buah bibir di sekolah karena berhasil meraih medali emas olimpiade matematika internasional.' Manakah pernyataan yang BENAR? (Jawaban benar lebih dari satu) ☐ A. Ungkapan 'buah bibir' bermakna bahan pembicaraan orang banyak ☐ B. Rian berprestasi dalam olimpiade matematika internasional ☐ C. Ungkapan 'kaki tangan' sesuai untuk prestasi gemilang Rian ☐ D. Prestasi Rian mengharumkan nama sekolahnya [Pilihan Ganda Kompleks: Jawaban benar lebih dari satu]</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -953,7 +997,11 @@
       <c r="H13" t="n">
         <v>60</v>
       </c>
-      <c r="I13" t="inlineStr"/>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -963,27 +1011,27 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 13: contoh soal pemahaman teks.</t>
+          <t>Kalimat utama paragraf yang membahas keindahan Pantai Parangtritis di Yogyakarta biasanya terletak di...</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. awal paragraf</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. tengah paragraf</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. akhir paragraf saja</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. bebas tanpa aturan</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -994,7 +1042,11 @@
       <c r="H14" t="n">
         <v>60</v>
       </c>
-      <c r="I14" t="inlineStr"/>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1004,27 +1056,27 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 14: contoh soal pemahaman teks.</t>
+          <t>Bagian formulir pendaftaran klub sains yang diisi dengan nama orang tua/wali siswa berfungsi untuk...</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. mengetahui izin dan penanggung jawab siswa</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. mengetahui hobi orang tua</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. menentukan alamat rumah guru</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. syarat bayar iuran bulanan</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1035,17 +1087,21 @@
       <c r="H15" t="n">
         <v>60</v>
       </c>
-      <c r="I15" t="inlineStr"/>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 15: contoh soal pemahaman teks.</t>
+          <t>Teks cerita fabel: 'Kura-kura yang tenang akhirnya memenangkan lomba lari melawan Kelinci yang sombong karena meremehkan lawan.' Tentukan kebenaran pernyataan berikut! [Pilihan Ganda Kompleks: Kategori Benar / Salah]</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1076,7 +1132,11 @@
       <c r="H16" t="n">
         <v>60</v>
       </c>
-      <c r="I16" t="inlineStr"/>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1086,27 +1146,27 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 16: contoh soal pemahaman teks.</t>
+          <t>Dalam cerita fiksi rakyat, tokoh antagonis adalah tokoh yang berwatak...</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. jahat atau penentang kebaikan</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. baik hati dan suka menolong</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. netral tanpa peran penting</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. bijaksana dan adil</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1117,7 +1177,11 @@
       <c r="H17" t="n">
         <v>60</v>
       </c>
-      <c r="I17" t="inlineStr"/>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1127,27 +1191,27 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 17: contoh soal pemahaman teks.</t>
+          <t>Ciri khas dari surat pribadi dibandingkan surat resmi adalah...</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. menggunakan bahasa santai dan tidak berformat kaku</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. menggunakan kop surat instansi resmi</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. ditandatangani kepala dinas</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. nomor surat dan lampiran wajib ada</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1158,17 +1222,21 @@
       <c r="H18" t="n">
         <v>60</v>
       </c>
-      <c r="I18" t="inlineStr"/>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 18: contoh soal pemahaman teks.</t>
+          <t>Perhatikan jadwal keberangkatan kereta: • Argo Bromo: 08.00 • Turangga: 14.30 • Bima: 17.15 Manakah pernyataan yang BENAR? (Jawaban benar lebih dari satu) ☐ A. Kereta Argo Bromo berangkat paling pagi pukul 08.00 ☐ B. Kereta Turangga berangkat pada siang menjelang sore hari ☐ C. Kereta Bima berangkat mendahului kereta Argo Bromo ☐ D. Ketiga jadwal kereta tersebut beroperasi pada hari yang sama [Pilihan Ganda Kompleks: Jawaban benar lebih dari satu]</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1199,7 +1267,11 @@
       <c r="H19" t="n">
         <v>60</v>
       </c>
-      <c r="I19" t="inlineStr"/>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1209,27 +1281,27 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 19: contoh soal pemahaman teks.</t>
+          <t>Ilmu yang mempelajari tentang fosil makhluk hidup purba disebut...</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>A. Pilihan A</t>
+          <t>A. palaeontologi</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>B. Pilihan B</t>
+          <t>B. arkeologi</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>C. Pilihan C</t>
+          <t>C. antropologi</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>D. Pilihan D</t>
+          <t>D. biologi</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1240,17 +1312,21 @@
       <c r="H20" t="n">
         <v>60</v>
       </c>
-      <c r="I20" t="inlineStr"/>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Multiple Choice</t>
+          <t>Multiple</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[Paket 10] Soal Bahasa 20: contoh soal pemahaman teks.</t>
+          <t>Fabel: 'Semut yang rajin mengumpulkan cadangan makanan berhasil selamat dari musim dingin, sementara Belalang yang malas kelaparan.' Tentukan kebenaran pernyataan berikut! [Pilihan Ganda Kompleks: Kategori Benar / Salah]</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1281,7 +1357,11 @@
       <c r="H21" t="n">
         <v>60</v>
       </c>
-      <c r="I21" t="inlineStr"/>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Pembahasan lengkap tersedia di modul teks.</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>